<commit_message>
Todas las modificaciones realizadas con la finalidad de implementar cambios al registro de Medidas de Protección. Se quedaron pendientes, con la finalidad de que en algún momento si se requiere retomarlos.
</commit_message>
<xml_diff>
--- a/format/medidasDeProteccion/documents/GeneratedFile.xlsx
+++ b/format/medidasDeProteccion/documents/GeneratedFile.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
-  <si>
-    <t>Periodo Correspondiente: 01-09-2025 AL 30-09-2025</t>
-  </si>
-  <si>
-    <t>Consultado: 30-09-2025</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="51">
+  <si>
+    <t>Periodo Correspondiente: 01-08-2025 AL 31-08-2025</t>
+  </si>
+  <si>
+    <t>Consultado: 28-10-2025</t>
   </si>
   <si>
     <t>Información Obtenida del Sistema Integral de Registro Estadístico (SIRE)</t>
@@ -123,6 +123,60 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Prueba Prueba Prueba</t>
+  </si>
+  <si>
+    <t>1003202520250</t>
+  </si>
+  <si>
+    <t>Homicidio calificado</t>
+  </si>
+  <si>
+    <t>Fiscalía Regional Morelia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+EJEMPLO DE VÍCTIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Masculino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+20 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Mexicana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Desconocido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Prohibición de acercarse o comunicarse con la víctima u ofendido
+Limitación para asistir o acercarse al domicilio de la víctima u ofendido o al lugar donde se encuentre
+Traslado de la víctima u ofendido a refugios o albergues temporales, así como de sus descendientes
+El reingreso de la víctima u ofendido a su domicilio, una vez que se salvaguarde su seguridad</t>
+  </si>
+  <si>
+    <t>2025-08-28 14:14:10</t>
+  </si>
+  <si>
+    <t>2025-08-28 14:13:00</t>
+  </si>
+  <si>
+    <t>2025-10-17 20:00:00</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Guardia Civil</t>
   </si>
 </sst>
 </file>
@@ -130,7 +184,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -145,8 +199,8 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="16"/>
-      <color rgb="000000"/>
+      <sz val="14"/>
+      <color rgb="FFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -154,8 +208,17 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="14"/>
-      <color rgb="FFFFFF"/>
+      <sz val="16"/>
+      <color rgb="000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -171,19 +234,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF"/>
+        <fgColor rgb="152f4a"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="152f4a"/>
+        <fgColor rgb="FFFFFF"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="18">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFF"/>
+      </top>
+    </border>
     <border>
       <left style="thin">
         <color rgb="152f4a"/>
@@ -239,6 +313,11 @@
       <top style="thin">
         <color rgb="FFFFFF"/>
       </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -258,15 +337,6 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFFFFF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFFFFF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFF"/>
-      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -295,9 +365,6 @@
       <top style="thin">
         <color rgb="FFFFFF"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
     </border>
     <border>
       <right style="thin">
@@ -320,69 +387,89 @@
         <color rgb="152f4a"/>
       </bottom>
     </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="12" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="13" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="14" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="15" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="16" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="12" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="13" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="14" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="17" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -779,7 +866,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AF10"/>
+  <dimension ref="A1:AF11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="7.2" customWidth="true" style="0"/>
@@ -817,418 +904,502 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32">
-      <c r="A1" s="1"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="14"/>
-      <c r="S1" s="14"/>
-      <c r="T1" s="14"/>
-      <c r="U1" s="14"/>
-      <c r="V1" s="14"/>
-      <c r="W1" s="14"/>
-      <c r="X1" s="14"/>
-      <c r="Y1" s="14"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="14"/>
-      <c r="AD1" s="14"/>
-      <c r="AE1" s="14"/>
-      <c r="AF1" s="15"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
+      <c r="X1" s="16"/>
+      <c r="Y1" s="16"/>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="5"/>
+      <c r="AB1" s="5"/>
+      <c r="AC1" s="16"/>
+      <c r="AD1" s="16"/>
+      <c r="AE1" s="16"/>
+      <c r="AF1" s="17"/>
     </row>
     <row r="2" spans="1:32">
-      <c r="A2" s="2"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="16"/>
-      <c r="U2" s="16"/>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="X2" s="16"/>
-      <c r="Y2" s="16"/>
-      <c r="Z2" s="5"/>
-      <c r="AA2" s="5"/>
-      <c r="AB2" s="5"/>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
-      <c r="AF2" s="17"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+      <c r="V2" s="18"/>
+      <c r="W2" s="18"/>
+      <c r="X2" s="18"/>
+      <c r="Y2" s="18"/>
+      <c r="Z2" s="6"/>
+      <c r="AA2" s="6"/>
+      <c r="AB2" s="6"/>
+      <c r="AC2" s="18"/>
+      <c r="AD2" s="18"/>
+      <c r="AE2" s="18"/>
+      <c r="AF2" s="19"/>
     </row>
     <row r="3" spans="1:32">
-      <c r="A3" s="2"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="16"/>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="5"/>
-      <c r="AA3" s="5"/>
-      <c r="AB3" s="5"/>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="17"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
+      <c r="V3" s="18"/>
+      <c r="W3" s="18"/>
+      <c r="X3" s="18"/>
+      <c r="Y3" s="18"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="18"/>
+      <c r="AD3" s="18"/>
+      <c r="AE3" s="18"/>
+      <c r="AF3" s="19"/>
     </row>
     <row r="4" spans="1:32">
-      <c r="A4" s="2"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="16"/>
-      <c r="W4" s="16"/>
-      <c r="X4" s="16"/>
-      <c r="Y4" s="16"/>
-      <c r="Z4" s="5"/>
-      <c r="AA4" s="5"/>
-      <c r="AB4" s="5"/>
-      <c r="AC4" s="16"/>
-      <c r="AD4" s="16"/>
-      <c r="AE4" s="16"/>
-      <c r="AF4" s="17"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="18"/>
+      <c r="W4" s="18"/>
+      <c r="X4" s="18"/>
+      <c r="Y4" s="18"/>
+      <c r="Z4" s="6"/>
+      <c r="AA4" s="6"/>
+      <c r="AB4" s="6"/>
+      <c r="AC4" s="18"/>
+      <c r="AD4" s="18"/>
+      <c r="AE4" s="18"/>
+      <c r="AF4" s="19"/>
     </row>
     <row r="5" spans="1:32">
-      <c r="A5" s="2"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5" t="s">
+      <c r="A5" s="3"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="16"/>
-      <c r="U5" s="16"/>
-      <c r="V5" s="16"/>
-      <c r="W5" s="16"/>
-      <c r="X5" s="16"/>
-      <c r="Y5" s="16"/>
-      <c r="Z5" s="5"/>
-      <c r="AA5" s="5"/>
-      <c r="AB5" s="5"/>
-      <c r="AC5" s="16"/>
-      <c r="AD5" s="16"/>
-      <c r="AE5" s="16"/>
-      <c r="AF5" s="17"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="18"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="6"/>
+      <c r="AA5" s="6"/>
+      <c r="AB5" s="6"/>
+      <c r="AC5" s="18"/>
+      <c r="AD5" s="18"/>
+      <c r="AE5" s="18"/>
+      <c r="AF5" s="19"/>
     </row>
     <row r="6" spans="1:32">
-      <c r="A6" s="2"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5" t="s">
+      <c r="A6" s="3"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
-      <c r="S6" s="16"/>
-      <c r="T6" s="16"/>
-      <c r="U6" s="16"/>
-      <c r="V6" s="16"/>
-      <c r="W6" s="16"/>
-      <c r="X6" s="16"/>
-      <c r="Y6" s="16"/>
-      <c r="Z6" s="5"/>
-      <c r="AA6" s="5"/>
-      <c r="AB6" s="5"/>
-      <c r="AC6" s="16"/>
-      <c r="AD6" s="16"/>
-      <c r="AE6" s="16"/>
-      <c r="AF6" s="17"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+      <c r="U6" s="18"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="6"/>
+      <c r="AA6" s="6"/>
+      <c r="AB6" s="6"/>
+      <c r="AC6" s="18"/>
+      <c r="AD6" s="18"/>
+      <c r="AE6" s="18"/>
+      <c r="AF6" s="19"/>
     </row>
     <row r="7" spans="1:32">
-      <c r="A7" s="2"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="16"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="16"/>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="5"/>
-      <c r="AA7" s="5"/>
-      <c r="AB7" s="5"/>
-      <c r="AC7" s="16"/>
-      <c r="AD7" s="16"/>
-      <c r="AE7" s="16"/>
-      <c r="AF7" s="17"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+      <c r="U7" s="18"/>
+      <c r="V7" s="18"/>
+      <c r="W7" s="18"/>
+      <c r="X7" s="18"/>
+      <c r="Y7" s="18"/>
+      <c r="Z7" s="6"/>
+      <c r="AA7" s="6"/>
+      <c r="AB7" s="6"/>
+      <c r="AC7" s="18"/>
+      <c r="AD7" s="18"/>
+      <c r="AE7" s="18"/>
+      <c r="AF7" s="19"/>
     </row>
     <row r="8" spans="1:32">
-      <c r="A8" s="3"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="18"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="18"/>
-      <c r="V8" s="18"/>
-      <c r="W8" s="18"/>
-      <c r="X8" s="18"/>
-      <c r="Y8" s="18"/>
-      <c r="Z8" s="6"/>
-      <c r="AA8" s="6"/>
-      <c r="AB8" s="6"/>
-      <c r="AC8" s="18"/>
-      <c r="AD8" s="18"/>
-      <c r="AE8" s="18"/>
-      <c r="AF8" s="19"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
+      <c r="T8" s="20"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20"/>
+      <c r="X8" s="20"/>
+      <c r="Y8" s="20"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="7"/>
+      <c r="AB8" s="7"/>
+      <c r="AC8" s="20"/>
+      <c r="AD8" s="20"/>
+      <c r="AE8" s="20"/>
+      <c r="AF8" s="21"/>
     </row>
     <row r="9" spans="1:32">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="9" t="s">
+      <c r="L9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M9" s="9" t="s">
+      <c r="M9" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="N9" s="9" t="s">
+      <c r="N9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9" t="s">
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11"/>
+      <c r="T9" s="11"/>
+      <c r="U9" s="11"/>
+      <c r="V9" s="11"/>
+      <c r="W9" s="11"/>
+      <c r="X9" s="11"/>
+      <c r="Y9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="Z9" s="9" t="s">
+      <c r="Z9" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="AA9" s="9" t="s">
+      <c r="AA9" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="AB9" s="9" t="s">
+      <c r="AB9" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="AC9" s="9" t="s">
+      <c r="AC9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="AD9" s="9"/>
-      <c r="AE9" s="9" t="s">
+      <c r="AD9" s="11"/>
+      <c r="AE9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="AF9" s="11" t="s">
+      <c r="AF9" s="13" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:32">
-      <c r="A10" s="8"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="P10" s="10" t="s">
+      <c r="P10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="Q10" s="10" t="s">
+      <c r="Q10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="R10" s="10" t="s">
+      <c r="R10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="10" t="s">
+      <c r="S10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="T10" s="10" t="s">
+      <c r="T10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="U10" s="10" t="s">
+      <c r="U10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="V10" s="10" t="s">
+      <c r="V10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="W10" s="10" t="s">
+      <c r="W10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="X10" s="10" t="s">
+      <c r="X10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="Y10" s="10"/>
-      <c r="Z10" s="10"/>
-      <c r="AA10" s="10"/>
-      <c r="AB10" s="10"/>
-      <c r="AC10" s="10" t="s">
+      <c r="Y10" s="1"/>
+      <c r="Z10" s="1"/>
+      <c r="AA10" s="1"/>
+      <c r="AB10" s="1"/>
+      <c r="AC10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AD10" s="10" t="s">
+      <c r="AD10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AE10" s="10"/>
-      <c r="AF10" s="12"/>
+      <c r="AE10" s="1"/>
+      <c r="AF10" s="14"/>
+    </row>
+    <row r="11" spans="1:32">
+      <c r="A11" s="10">
+        <v>7729</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="22">
+        <v>4567</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H11" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="K11" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="M11" s="22">
+        <v>4</v>
+      </c>
+      <c r="N11" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="O11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q11" s="22"/>
+      <c r="R11" s="22"/>
+      <c r="S11" s="22"/>
+      <c r="T11" s="22"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="22"/>
+      <c r="W11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="X11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y11" s="22">
+        <v>60</v>
+      </c>
+      <c r="Z11" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA11" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB11" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC11" s="22"/>
+      <c r="AD11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE11" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF11" s="23" t="s">
+        <v>50</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>